<commit_message>
Updates after a while
</commit_message>
<xml_diff>
--- a/info/key_markers.xlsx
+++ b/info/key_markers.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mgierlinski/Work/Projects/BetaReg/BetaReg_ST/info/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA5D15E5-DA8A-8A49-AF6C-8978E3F83598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ABA8118-A819-8543-80B3-69103C504970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10620" yWindow="2500" windowWidth="27640" windowHeight="16940" xr2:uid="{3297E706-06BE-2746-B04B-E4FC657513D2}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="62">
   <si>
     <t>MPC</t>
   </si>
@@ -189,6 +189,39 @@
   </si>
   <si>
     <t>HBA2</t>
+  </si>
+  <si>
+    <t>Ductal</t>
+  </si>
+  <si>
+    <t>Acinar</t>
+  </si>
+  <si>
+    <t>SLC4A4</t>
+  </si>
+  <si>
+    <t>ANXA4</t>
+  </si>
+  <si>
+    <t>CFTR</t>
+  </si>
+  <si>
+    <t>CPA1</t>
+  </si>
+  <si>
+    <t>PRSS1</t>
+  </si>
+  <si>
+    <t>CLPS</t>
+  </si>
+  <si>
+    <t>Ductoacinar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CFTR </t>
+  </si>
+  <si>
+    <t>HES6</t>
   </si>
 </sst>
 </file>
@@ -568,10 +601,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9F179BB-D4EE-6E44-8D12-1CE86B57DE2D}">
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:Q45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>24</v>
       </c>
@@ -614,8 +647,17 @@
       <c r="N1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O1" t="s">
+        <v>51</v>
+      </c>
+      <c r="P1" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -623,7 +665,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -631,7 +673,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -639,7 +681,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -647,7 +689,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -655,7 +697,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -663,7 +705,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -671,7 +713,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -679,7 +721,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -687,7 +729,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -701,7 +743,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -712,7 +754,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -726,7 +768,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -737,7 +779,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -745,7 +787,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -884,7 +926,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>45</v>
       </c>
@@ -892,7 +934,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>47</v>
       </c>
@@ -900,7 +942,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>48</v>
       </c>
@@ -908,7 +950,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>49</v>
       </c>
@@ -916,11 +958,75 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>50</v>
       </c>
       <c r="N37" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>53</v>
+      </c>
+      <c r="O38" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>54</v>
+      </c>
+      <c r="O39" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>55</v>
+      </c>
+      <c r="O40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>56</v>
+      </c>
+      <c r="P41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>57</v>
+      </c>
+      <c r="P42" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>58</v>
+      </c>
+      <c r="P43" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q45" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>